<commit_message>
Add provider portal with auction-based loan offers; fix disbursement race and admin archive-tab bugs
Adds a full Provider role (login, dashboard, models, migrations 020-023) that
lets lending providers submit loan offers on approved applications and
schedule property valuations. Also folds in a batch of testing-session fixes:
a double-disbursement race in LoanDisbursement.confirmScheduledDisbursement,
an always-false showArchived check that left admins' Archived health-report
tab permanently empty, AuthContext SIGNED_IN de-dup and dev-only logging, plus
wizard/admin/support UI polish and an ML model retrain.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/e-Rumah_Testing_Verification_Checklist.xlsx
+++ b/e-Rumah_Testing_Verification_Checklist.xlsx
@@ -1444,11 +1444,19 @@
       </c>
       <c r="F5" s="48" t="inlineStr">
         <is>
-          <t>Not Tested</t>
-        </is>
-      </c>
-      <c r="G5" s="49" t="n"/>
-      <c r="H5" s="48" t="n"/>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="G5" s="49" t="inlineStr">
+        <is>
+          <t>Code-verified: PDF/JPG/PNG/WEBP &lt;=10MB validated via file picker and drag-drop. But JPG/PNG are never stored natively - the view forces a window.confirm to convert images to PDF first (convertImagesToPDF); declining the conversion aborts the upload entirely.</t>
+        </is>
+      </c>
+      <c r="H5" s="48" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
       <c r="I5" s="48" t="n"/>
     </row>
     <row r="6" ht="48.75" customHeight="1" s="27">
@@ -1522,11 +1530,19 @@
       </c>
       <c r="F7" s="48" t="inlineStr">
         <is>
-          <t>Not Tested</t>
-        </is>
-      </c>
-      <c r="G7" s="49" t="n"/>
-      <c r="H7" s="48" t="n"/>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="G7" s="49" t="inlineStr">
+        <is>
+          <t>Code-verified: HealthReport.getByUser filters to the logged-in elder's own reports only; title/type/report date/status render. No 'due date' column is shown in the list - due_status is only used internally for tab filtering.</t>
+        </is>
+      </c>
+      <c r="H7" s="48" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
       <c r="I7" s="48" t="n"/>
     </row>
     <row r="8" ht="33.75" customHeight="1" s="27">
@@ -1557,11 +1573,19 @@
       </c>
       <c r="F8" s="50" t="inlineStr">
         <is>
-          <t>Not Tested</t>
-        </is>
-      </c>
-      <c r="G8" s="51" t="n"/>
-      <c r="H8" s="50" t="n"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G8" s="51" t="inlineStr">
+        <is>
+          <t>Code-verified: search matches report title and provider_name client-side; Clear Search resets and restores the full list.</t>
+        </is>
+      </c>
+      <c r="H8" s="50" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
       <c r="I8" s="50" t="n"/>
     </row>
     <row r="9" ht="48.75" customHeight="1" s="27">
@@ -1592,11 +1616,19 @@
       </c>
       <c r="F9" s="48" t="inlineStr">
         <is>
-          <t>Not Tested</t>
-        </is>
-      </c>
-      <c r="G9" s="49" t="n"/>
-      <c r="H9" s="48" t="n"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G9" s="49" t="inlineStr">
+        <is>
+          <t>Code-verified: report-type/date-range filters combine with upload/due-status tab filters in one pipeline; Clear Filters resets search+filters+tab together.</t>
+        </is>
+      </c>
+      <c r="H9" s="48" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
       <c r="I9" s="48" t="n"/>
     </row>
     <row r="10" ht="48.75" customHeight="1" s="27">
@@ -1627,11 +1659,19 @@
       </c>
       <c r="F10" s="50" t="inlineStr">
         <is>
-          <t>Not Tested</t>
-        </is>
-      </c>
-      <c r="G10" s="51" t="n"/>
-      <c r="H10" s="50" t="n"/>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="G10" s="51" t="inlineStr">
+        <is>
+          <t>Code-verified: sort dropdown only offers Report Date/Upload Date/Title/Type/Status - no 'healthcare provider' or 'due date' sort option in the UI, though the model would accept those columns. Asc/desc toggle works for the available fields.</t>
+        </is>
+      </c>
+      <c r="H10" s="50" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
       <c r="I10" s="50" t="n"/>
     </row>
     <row r="11" ht="33.75" customHeight="1" s="27">
@@ -1791,11 +1831,19 @@
       </c>
       <c r="F14" s="50" t="inlineStr">
         <is>
-          <t>Not Tested</t>
-        </is>
-      </c>
-      <c r="G14" s="51" t="n"/>
-      <c r="H14" s="50" t="n"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G14" s="51" t="inlineStr">
+        <is>
+          <t>Code-verified: shareViaEmail sends an email with the share link + expiry date via an edge function; downloadHealthReportFile independently fetches and downloads the report as a file.</t>
+        </is>
+      </c>
+      <c r="H14" s="50" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
       <c r="I14" s="50" t="n"/>
     </row>
     <row r="15" ht="33.75" customHeight="1" s="27">
@@ -1869,11 +1917,19 @@
       </c>
       <c r="F16" s="50" t="inlineStr">
         <is>
-          <t>Not Tested</t>
-        </is>
-      </c>
-      <c r="G16" s="51" t="n"/>
-      <c r="H16" s="50" t="n"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G16" s="51" t="inlineStr">
+        <is>
+          <t>Code-verified: archive_old_health_reports() only flips health_report_status to Archived - it never deletes storage objects or DB rows, so report_file_url stays valid indefinitely.</t>
+        </is>
+      </c>
+      <c r="H16" s="50" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
       <c r="I16" s="50" t="n"/>
     </row>
     <row r="17" ht="33.75" customHeight="1" s="27">
@@ -1904,11 +1960,19 @@
       </c>
       <c r="F17" s="48" t="inlineStr">
         <is>
-          <t>Not Tested</t>
-        </is>
-      </c>
-      <c r="G17" s="49" t="n"/>
-      <c r="H17" s="48" t="n"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G17" s="49" t="inlineStr">
+        <is>
+          <t>Code-verified: /admin/health-reports queries admin_health_report_view with no user_id filter and attaches each report's owner name/email.</t>
+        </is>
+      </c>
+      <c r="H17" s="48" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
       <c r="I17" s="48" t="n"/>
     </row>
     <row r="18" ht="48.75" customHeight="1" s="27">
@@ -1939,11 +2003,19 @@
       </c>
       <c r="F18" s="50" t="inlineStr">
         <is>
-          <t>Not Tested</t>
-        </is>
-      </c>
-      <c r="G18" s="51" t="n"/>
-      <c r="H18" s="50" t="n"/>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="G18" s="51" t="inlineStr">
+        <is>
+          <t>Code-verified: admin search covers report_type/title/notes/user name/email/IC/phone but NOT provider_name (missing from both server and client-side search) despite the requirement naming provider-name search. Sort has the same gaps as HM-06 (no provider/due-date option).</t>
+        </is>
+      </c>
+      <c r="H18" s="50" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
       <c r="I18" s="50" t="n"/>
     </row>
     <row r="19" ht="33.75" customHeight="1" s="27">
@@ -1974,11 +2046,19 @@
       </c>
       <c r="F19" s="48" t="inlineStr">
         <is>
-          <t>Not Tested</t>
-        </is>
-      </c>
-      <c r="G19" s="49" t="n"/>
-      <c r="H19" s="48" t="n"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G19" s="49" t="inlineStr">
+        <is>
+          <t>Code-verified: admin opens PDF viewer, clicks Approve, confirms in a modal, then approveHealthReport sets status to Reviewed; elder's next fetch reflects it.</t>
+        </is>
+      </c>
+      <c r="H19" s="48" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
       <c r="I19" s="48" t="n"/>
     </row>
     <row r="20" ht="48.75" customHeight="1" s="27">
@@ -2009,11 +2089,19 @@
       </c>
       <c r="F20" s="50" t="inlineStr">
         <is>
-          <t>Not Tested</t>
-        </is>
-      </c>
-      <c r="G20" s="51" t="n"/>
-      <c r="H20" s="50" t="n"/>
+          <t>Pass (fixed this session)</t>
+        </is>
+      </c>
+      <c r="G20" s="51" t="inlineStr">
+        <is>
+          <t>Bug found &amp; fixed: showArchived option was computed as `activeTab==='archived' &amp;&amp; userRole!=='admin'`, which is always false for admin - so an admin's Archived tab always fetched with archived reports excluded and rendered permanently empty. Fixed by dropping the role condition so any role can view the Archived tab. Confirmation-before-archive modal already worked correctly.</t>
+        </is>
+      </c>
+      <c r="H20" s="50" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
       <c r="I20" s="50" t="n"/>
     </row>
     <row r="21" ht="48.75" customHeight="1" s="27">
@@ -2044,11 +2132,19 @@
       </c>
       <c r="F21" s="48" t="inlineStr">
         <is>
-          <t>Not Tested</t>
-        </is>
-      </c>
-      <c r="G21" s="49" t="n"/>
-      <c r="H21" s="48" t="n"/>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="G21" s="49" t="inlineStr">
+        <is>
+          <t>Code-verified: flagging is blocked until a reason is entered (client+server); flagged reports are routed into the Customer Support dashboard queue (HealthReport.getFlagged). Elder 'notification' is passive only - a banner appears next time they open the report; there is no push/email notification sent to the elder.</t>
+        </is>
+      </c>
+      <c r="H21" s="48" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
       <c r="I21" s="48" t="n"/>
     </row>
     <row r="22" ht="33.75" customHeight="1" s="27">
@@ -2079,11 +2175,19 @@
       </c>
       <c r="F22" s="50" t="inlineStr">
         <is>
-          <t>Not Tested</t>
-        </is>
-      </c>
-      <c r="G22" s="51" t="n"/>
-      <c r="H22" s="50" t="n"/>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="G22" s="51" t="inlineStr">
+        <is>
+          <t>Code-verified: due_status (Overdue/Due Soon/Up to Date) is computed daily and drives the tab filters correctly, but the results-table badge always renders health_report_status (Pending/Reviewed/Flagged/Archived) - due_status is never shown as a per-row badge, and StatusBadge has no CSS classes for Overdue/Due Soon states at all. This is a UI/design gap (a distinct due-status badge column would need to be added), not a one-line bug - left as a follow-up rather than building new UI unasked.</t>
+        </is>
+      </c>
+      <c r="H22" s="50" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
       <c r="I22" s="50" t="n"/>
     </row>
     <row r="23" ht="48.75" customHeight="1" s="27">
@@ -2114,11 +2218,19 @@
       </c>
       <c r="F23" s="48" t="inlineStr">
         <is>
-          <t>Not Tested</t>
-        </is>
-      </c>
-      <c r="G23" s="49" t="n"/>
-      <c r="H23" s="48" t="n"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G23" s="49" t="inlineStr">
+        <is>
+          <t>Code-verified: create/edit/mark-notified/delete a reminder all persist via Supabase; every mutation handler reloads reminders/upcoming/overdue lists afterward.</t>
+        </is>
+      </c>
+      <c r="H23" s="48" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
       <c r="I23" s="48" t="n"/>
     </row>
   </sheetData>
@@ -2266,11 +2378,19 @@
       </c>
       <c r="F5" s="48" t="inlineStr">
         <is>
-          <t>Not Tested</t>
-        </is>
-      </c>
-      <c r="G5" s="49" t="n"/>
-      <c r="H5" s="48" t="n"/>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="G5" s="49" t="inlineStr">
+        <is>
+          <t>Code-verified: all 7 steps exist, are sequentially navigable, and a visible progress bar/'Step X of 7' indicator is shown. However there is no 'select lending organisation' step - the scheme is hardcoded to a single generic placeholder - and the actual step titles/content don't match the described breakdown (e.g. step 5 is 'Privacy, Documents &amp; Declaration', step 6 is 'Acknowledgement Form').</t>
+        </is>
+      </c>
+      <c r="H5" s="48" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
       <c r="I5" s="48" t="n"/>
     </row>
     <row r="6" ht="48.75" customHeight="1" s="27">
@@ -2344,11 +2464,19 @@
       </c>
       <c r="F7" s="48" t="inlineStr">
         <is>
-          <t>Not Tested</t>
-        </is>
-      </c>
-      <c r="G7" s="49" t="n"/>
-      <c r="H7" s="48" t="n"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G7" s="49" t="inlineStr">
+        <is>
+          <t>Code-verified: validateAge blocks age &lt;55 and &gt;120 with clear messages; parseICNumber derives birth date and sex from the Malaysian IC and auto-fills DOB, re-validated in validateStep1.</t>
+        </is>
+      </c>
+      <c r="H7" s="48" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
       <c r="I7" s="48" t="n"/>
     </row>
     <row r="8" ht="48.75" customHeight="1" s="27">
@@ -2379,11 +2507,19 @@
       </c>
       <c r="F8" s="50" t="inlineStr">
         <is>
-          <t>Not Tested</t>
-        </is>
-      </c>
-      <c r="G8" s="51" t="n"/>
-      <c r="H8" s="50" t="n"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G8" s="51" t="inlineStr">
+        <is>
+          <t>Code-verified: no &lt;form&gt; element exists in the wizard (no native-submit path, no required=/pattern= HTML attributes anywhere); handleNext is a plain button handler blocked by custom validateStep with field-specific messages for IC/phone/postcode/email/account number.</t>
+        </is>
+      </c>
+      <c r="H8" s="50" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
       <c r="I8" s="50" t="n"/>
     </row>
     <row r="9" ht="48.75" customHeight="1" s="27">
@@ -2414,11 +2550,19 @@
       </c>
       <c r="F9" s="48" t="inlineStr">
         <is>
-          <t>Not Tested</t>
-        </is>
-      </c>
-      <c r="G9" s="49" t="n"/>
-      <c r="H9" s="48" t="n"/>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="G9" s="49" t="inlineStr">
+        <is>
+          <t>Code-verified: encumbrance, excluded KL postcodes, and insufficient leasehold remaining-lease (&lt;90 years) all correctly block submission with messages. But 'unsupported property type' is not actually a disqualifying check (property type is a free choice with no eligibility logic), and non-freehold tenure alone isn't disqualifying (only insufficient lease-years is).</t>
+        </is>
+      </c>
+      <c r="H9" s="48" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
       <c r="I9" s="48" t="n"/>
     </row>
     <row r="10" ht="78.75" customHeight="1" s="27">
@@ -2492,11 +2636,19 @@
       </c>
       <c r="F11" s="48" t="inlineStr">
         <is>
-          <t>Not Tested</t>
-        </is>
-      </c>
-      <c r="G11" s="49" t="n"/>
-      <c r="H11" s="48" t="n"/>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="G11" s="49" t="inlineStr">
+        <is>
+          <t>Code-verified: Maintain Application page supports document re-upload for missing/flagged docs, termination request, PDF download, and links out to a separate nominee-edit route. There is no personal-details or property-details edit capability anywhere on this page - those fields are only writable during original wizard submission.</t>
+        </is>
+      </c>
+      <c r="H11" s="48" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
       <c r="I11" s="48" t="n"/>
     </row>
     <row r="12" ht="33.75" customHeight="1" s="27">
@@ -2613,11 +2765,19 @@
       </c>
       <c r="F14" s="50" t="inlineStr">
         <is>
-          <t>Not Tested</t>
-        </is>
-      </c>
-      <c r="G14" s="51" t="n"/>
-      <c r="H14" s="50" t="n"/>
+          <t>Pass*</t>
+        </is>
+      </c>
+      <c r="G14" s="51" t="inlineStr">
+        <is>
+          <t>Code-verified: current status and an accurate timeline (submitted/reviewed/approved/termination events) built from real timestamps are always rendered. Caveat: the 'draft' stage is never actually reached on this page by design - ProtectedRoute redirects incomplete-status users straight to the wizard instead.</t>
+        </is>
+      </c>
+      <c r="H14" s="50" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
       <c r="I14" s="50" t="n"/>
     </row>
     <row r="15" ht="48.75" customHeight="1" s="27">
@@ -2691,11 +2851,19 @@
       </c>
       <c r="F16" s="50" t="inlineStr">
         <is>
-          <t>Not Tested</t>
-        </is>
-      </c>
-      <c r="G16" s="51" t="n"/>
-      <c r="H16" s="50" t="n"/>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="G16" s="51" t="inlineStr">
+        <is>
+          <t>Not implemented: no code anywhere creates a nominee-initiated redemption application, links one to an original application, or exposes a 'deceased/terminated scheme' redemption concept. Nominee.js only exposes get/update/search operations, nothing resembling this feature.</t>
+        </is>
+      </c>
+      <c r="H16" s="50" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
       <c r="I16" s="50" t="n"/>
     </row>
     <row r="17" ht="33.75" customHeight="1" s="27">
@@ -2769,11 +2937,19 @@
       </c>
       <c r="F18" s="50" t="inlineStr">
         <is>
-          <t>Not Tested</t>
-        </is>
-      </c>
-      <c r="G18" s="51" t="n"/>
-      <c r="H18" s="50" t="n"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G18" s="51" t="inlineStr">
+        <is>
+          <t>Code-verified: handleFileUpload/handleFileDelete correctly mutate formData.documents[type] (delete resets, upload overwrites) and the upload UI only renders when no document is attached, so only the final document is ever referenced. Caveat: this happens on Steps 1 and 3 in the current wizard, not a distinct 'Step 6' as the test description assumes.</t>
+        </is>
+      </c>
+      <c r="H18" s="50" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
       <c r="I18" s="50" t="n"/>
     </row>
     <row r="19" ht="48.75" customHeight="1" s="27">
@@ -3050,11 +3226,19 @@
       </c>
       <c r="F5" s="48" t="inlineStr">
         <is>
-          <t>Not Tested</t>
-        </is>
-      </c>
-      <c r="G5" s="49" t="n"/>
-      <c r="H5" s="48" t="n"/>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="G5" s="49" t="inlineStr">
+        <is>
+          <t>Code-verified: the FAQ accordion covers post-signup obligations/inheritance/divorce scenarios, but does not include 'required documents' as FAQ content, and payout calculation/eligibility appear elsewhere (a separate info card) rather than as FAQ entries - not all four required topics are covered as FAQ content.</t>
+        </is>
+      </c>
+      <c r="H5" s="48" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
       <c r="I5" s="48" t="n"/>
     </row>
     <row r="6" ht="33.75" customHeight="1" s="27">
@@ -3085,11 +3269,19 @@
       </c>
       <c r="F6" s="50" t="inlineStr">
         <is>
-          <t>Not Tested</t>
-        </is>
-      </c>
-      <c r="G6" s="51" t="n"/>
-      <c r="H6" s="50" t="n"/>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="G6" s="51" t="inlineStr">
+        <is>
+          <t>Not implemented: no guided tutorial/walkthrough component exists for the application wizard or health-report upload. The closest content (StepByStep 'How To Apply') describes an offline legacy process (visiting EPF/AKPK branches) that contradicts the actual online wizard.</t>
+        </is>
+      </c>
+      <c r="H6" s="50" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
       <c r="I6" s="50" t="n"/>
     </row>
     <row r="7" ht="48.75" customHeight="1" s="27">
@@ -3163,11 +3355,19 @@
       </c>
       <c r="F8" s="50" t="inlineStr">
         <is>
-          <t>Not Tested</t>
-        </is>
-      </c>
-      <c r="G8" s="51" t="n"/>
-      <c r="H8" s="50" t="n"/>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="G8" s="51" t="inlineStr">
+        <is>
+          <t>Code-verified: phone and email are stored via settingsService (localStorage) and displayed to the elder on the support page, and update/reload correctly. No 'operating hours' field exists anywhere in settingsService or its consumers - only email/phone are implemented.</t>
+        </is>
+      </c>
+      <c r="H8" s="50" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
       <c r="I8" s="50" t="n"/>
     </row>
     <row r="9" ht="48.75" customHeight="1" s="27">
@@ -3198,11 +3398,19 @@
       </c>
       <c r="F9" s="48" t="inlineStr">
         <is>
-          <t>Not Tested</t>
-        </is>
-      </c>
-      <c r="G9" s="49" t="n"/>
-      <c r="H9" s="48" t="n"/>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="G9" s="49" t="inlineStr">
+        <is>
+          <t>Code-verified: the flagged-document alert is real (a banner on the Maintain Application page). A deadline-approaching alert only exists as a passive 'Upcoming Reminders' list entry tied to user-created health-check reminders, not an application/document deadline, and it's a dashboard list item rather than a pushed alert; Notification.js is an empty stub confirming no real alert infrastructure exists.</t>
+        </is>
+      </c>
+      <c r="H9" s="48" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
       <c r="I9" s="48" t="n"/>
     </row>
     <row r="10" ht="48.75" customHeight="1" s="27">
@@ -3233,11 +3441,19 @@
       </c>
       <c r="F10" s="50" t="inlineStr">
         <is>
-          <t>Not Tested</t>
-        </is>
-      </c>
-      <c r="G10" s="51" t="n"/>
-      <c r="H10" s="50" t="n"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G10" s="51" t="inlineStr">
+        <is>
+          <t>Code-verified: staff dashboard lists inquiries and groups them via a status dropdown (All/Open/In Progress/Resolved) plus category tabs (Inquiries/Nominees/Health Report).</t>
+        </is>
+      </c>
+      <c r="H10" s="50" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
       <c r="I10" s="50" t="n"/>
     </row>
     <row r="11" ht="48.75" customHeight="1" s="27">
@@ -3397,11 +3613,19 @@
       </c>
       <c r="F14" s="50" t="inlineStr">
         <is>
-          <t>Not Tested</t>
-        </is>
-      </c>
-      <c r="G14" s="51" t="n"/>
-      <c r="H14" s="50" t="n"/>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="G14" s="51" t="inlineStr">
+        <is>
+          <t>Not implemented: no compose/broadcast capability exists anywhere. SupportConversation.send() only appends a message to an already-existing inquiry/nominee/health-report thread - there is no code path to message an arbitrary elder or a group.</t>
+        </is>
+      </c>
+      <c r="H14" s="50" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
       <c r="I14" s="50" t="n"/>
     </row>
     <row r="15" ht="33.75" customHeight="1" s="27">
@@ -3432,11 +3656,19 @@
       </c>
       <c r="F15" s="48" t="inlineStr">
         <is>
-          <t>Not Tested</t>
-        </is>
-      </c>
-      <c r="G15" s="49" t="n"/>
-      <c r="H15" s="48" t="n"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G15" s="49" t="inlineStr">
+        <is>
+          <t>Code-verified: staff edits validate and persist to localStorage via settingsService; the elder support page reloads and picks up new values on mount, with a bonus cross-tab storage-event sync.</t>
+        </is>
+      </c>
+      <c r="H15" s="48" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
       <c r="I15" s="48" t="n"/>
     </row>
     <row r="16" ht="48.75" customHeight="1" s="27">
@@ -3467,11 +3699,19 @@
       </c>
       <c r="F16" s="50" t="inlineStr">
         <is>
-          <t>Not Tested</t>
-        </is>
-      </c>
-      <c r="G16" s="51" t="n"/>
-      <c r="H16" s="50" t="n"/>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="G16" s="51" t="inlineStr">
+        <is>
+          <t>Code-verified: the staff-side flow works end to end - nominee details render fully and flagging an application (with a reason) correctly sets is_flagged/flagged_reason/flagged_code on the application. But nothing in the admin controllers/views reads these fields - the flag never actually surfaces to the administrator, a gap distinct from (and in addition to) the separate AD-08 nominee-approve/reject gap.</t>
+        </is>
+      </c>
+      <c r="H16" s="50" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
       <c r="I16" s="50" t="n"/>
     </row>
     <row r="17" ht="48.75" customHeight="1" s="27">
@@ -3502,11 +3742,19 @@
       </c>
       <c r="F17" s="48" t="inlineStr">
         <is>
-          <t>Not Tested</t>
-        </is>
-      </c>
-      <c r="G17" s="49" t="n"/>
-      <c r="H17" s="48" t="n"/>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="G17" s="49" t="inlineStr">
+        <is>
+          <t>Code-verified: HealthReport.getFlagged() is called and flagged health reports are merged into the support dashboard's queue. However the actual flagged_reason field is never rendered anywhere in the detail panel - only a generic 'notes' field is shown - so the flag reason itself doesn't reach the queue's UI.</t>
+        </is>
+      </c>
+      <c r="H17" s="48" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
       <c r="I17" s="48" t="n"/>
     </row>
     <row r="18" ht="33.75" customHeight="1" s="27">
@@ -3537,11 +3785,19 @@
       </c>
       <c r="F18" s="50" t="inlineStr">
         <is>
-          <t>Not Tested</t>
-        </is>
-      </c>
-      <c r="G18" s="51" t="n"/>
-      <c r="H18" s="50" t="n"/>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="G18" s="51" t="inlineStr">
+        <is>
+          <t>Code-verified: sort and the status filter both work correctly. But the search box is dead code - handleSearch/searchTerm are passed as props but never wired to any input element, so staff cannot actually search inquiries despite Inquiry.search() existing in the model; the filterField (status vs priority) toggle also has no UI control.</t>
+        </is>
+      </c>
+      <c r="H18" s="50" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
       <c r="I18" s="50" t="n"/>
     </row>
   </sheetData>
@@ -6110,8 +6366,16 @@
           <t>Not Tested</t>
         </is>
       </c>
-      <c r="G17" s="49" t="n"/>
-      <c r="H17" s="48" t="n"/>
+      <c r="G17" s="49" t="inlineStr">
+        <is>
+          <t>Not code-verifiable in a meaningful way - touch-target size and readability across desktop+mobile viewports need an actual visual review. Directional note: some secondary UI chrome (admin badges/labels) uses fonts as small as 11-13px (see NF-05's font finding), but primary user-facing forms were not measured. Left as Not Tested pending a live pass.</t>
+        </is>
+      </c>
+      <c r="H17" s="48" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
       <c r="I17" s="48" t="n"/>
     </row>
     <row r="18" ht="33.75" customHeight="1" s="27">

</xml_diff>